<commit_message>
Actualizacion completa: auditor de validaciones, estilos, vistas y plantillas
</commit_message>
<xml_diff>
--- a/REPORTE MENSUAL REQUERIMIENTOS.xlsx
+++ b/REPORTE MENSUAL REQUERIMIENTOS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\52553\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jose Angel\Desktop\Tablero_pemex11\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA3A2815-4C84-46CB-A39C-C2797AF06E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A5AAE14-C4F6-4C6E-8964-340A3D622956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D60847B7-BCF7-432B-BE25-7AAD2B4F7A5B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="2" xr2:uid="{D60847B7-BCF7-432B-BE25-7AAD2B4F7A5B}"/>
   </bookViews>
   <sheets>
     <sheet name="ACTIVOS" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5536" uniqueCount="760">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5554" uniqueCount="762">
   <si>
     <t>#</t>
   </si>
@@ -2609,11 +2609,20 @@
   <si>
     <t>Recepción básica del SIGPPSC</t>
   </si>
+  <si>
+    <t xml:space="preserve">DCF0119 52720 Reporte de Saldos </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DCF0079 13720 Reporte de Saldos </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2649,20 +2658,54 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="58">
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -2701,7 +2744,64 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -2737,100 +2837,10 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2942,30 +2952,30 @@
   <autoFilter ref="A1:AA100" xr:uid="{5912A661-203D-4C9C-9CB5-42BFA11CDC54}"/>
   <tableColumns count="27">
     <tableColumn id="1" xr3:uid="{4D22CF92-EDC8-4CA7-BA1E-D4C177B0E7F5}" uniqueName="1" name="#" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{EFF7F135-8BF8-440B-825B-21DC2AF85F6D}" uniqueName="2" name="Estado" queryTableFieldId="2" dataDxfId="57"/>
-    <tableColumn id="3" xr3:uid="{13155E22-50B1-4878-A267-F021291C50B0}" uniqueName="3" name="Grupo de tarea" queryTableFieldId="3" dataDxfId="56"/>
-    <tableColumn id="4" xr3:uid="{44555AAD-1162-4323-A10E-C671C766E1C3}" uniqueName="4" name="Asunto" queryTableFieldId="4" dataDxfId="55"/>
-    <tableColumn id="5" xr3:uid="{378F2931-3BF9-446D-8EA3-563566003DFF}" uniqueName="5" name="Situación actual" queryTableFieldId="5" dataDxfId="54"/>
-    <tableColumn id="6" xr3:uid="{3E21B045-28B0-4EE9-8BC5-90D8D60F35F7}" uniqueName="6" name="Impacto de Otros Proyectos" queryTableFieldId="6" dataDxfId="53"/>
-    <tableColumn id="7" xr3:uid="{0FF46444-B59C-4CEC-8AAA-D66A27A7DBFA}" uniqueName="7" name="Capacidades" queryTableFieldId="7" dataDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{4B9F5718-E3BA-4D72-9EFE-BC7C9F418A1A}" uniqueName="8" name="Acciones Coordinadas STI" queryTableFieldId="8" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{EFF7F135-8BF8-440B-825B-21DC2AF85F6D}" uniqueName="2" name="Estado" queryTableFieldId="2" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{13155E22-50B1-4878-A267-F021291C50B0}" uniqueName="3" name="Grupo de tarea" queryTableFieldId="3" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{44555AAD-1162-4323-A10E-C671C766E1C3}" uniqueName="4" name="Asunto" queryTableFieldId="4" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{378F2931-3BF9-446D-8EA3-563566003DFF}" uniqueName="5" name="Situación actual" queryTableFieldId="5" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{3E21B045-28B0-4EE9-8BC5-90D8D60F35F7}" uniqueName="6" name="Impacto de Otros Proyectos" queryTableFieldId="6" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{0FF46444-B59C-4CEC-8AAA-D66A27A7DBFA}" uniqueName="7" name="Capacidades" queryTableFieldId="7" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{4B9F5718-E3BA-4D72-9EFE-BC7C9F418A1A}" uniqueName="8" name="Acciones Coordinadas STI" queryTableFieldId="8" dataDxfId="49"/>
     <tableColumn id="9" xr3:uid="{BAA65803-EA5A-4D7F-8822-2C924A847560}" uniqueName="9" name="% Planeado" queryTableFieldId="9"/>
     <tableColumn id="10" xr3:uid="{A6A80147-E0C7-4FC8-9A6B-66E5C7BD334D}" uniqueName="10" name="% Ponderado" queryTableFieldId="10"/>
-    <tableColumn id="11" xr3:uid="{A4D2FA40-7BFE-4BD0-8ABC-D3B5B6E1F880}" uniqueName="11" name="Asignado a" queryTableFieldId="11" dataDxfId="50"/>
-    <tableColumn id="12" xr3:uid="{A35DA601-AB84-43F1-9914-8079DAD3A955}" uniqueName="12" name="Clasificación requerimiento" queryTableFieldId="12" dataDxfId="49"/>
-    <tableColumn id="13" xr3:uid="{C9B9BAF0-055B-416F-A5B2-65E763015FD7}" uniqueName="13" name="Subdirección solicitante" queryTableFieldId="13" dataDxfId="48"/>
-    <tableColumn id="14" xr3:uid="{BC3DDA39-962F-4573-996E-77BD8BE40FB6}" uniqueName="14" name="Prioridad Origen" queryTableFieldId="14" dataDxfId="47"/>
-    <tableColumn id="15" xr3:uid="{8BE5F5D0-62C5-4ABC-BF0B-A948639C8D12}" uniqueName="15" name="F.Inicio base" queryTableFieldId="15" dataDxfId="46"/>
-    <tableColumn id="16" xr3:uid="{390C035A-E22A-4A22-8A40-84D899F95E4B}" uniqueName="16" name="F. fin base" queryTableFieldId="16" dataDxfId="45"/>
-    <tableColumn id="17" xr3:uid="{7A05EABF-0116-4EB6-8560-5EBF9F6F108B}" uniqueName="17" name="Fase" queryTableFieldId="17" dataDxfId="44"/>
-    <tableColumn id="18" xr3:uid="{7EF58F9F-F423-4B0E-AAC3-480E0531EF0C}" uniqueName="18" name="Edo. Salud" queryTableFieldId="18" dataDxfId="43"/>
-    <tableColumn id="19" xr3:uid="{A62386F7-0F54-49A2-86AC-75CB742CADA8}" uniqueName="19" name="Área Responsable Habilitación" queryTableFieldId="19" dataDxfId="42"/>
+    <tableColumn id="11" xr3:uid="{A4D2FA40-7BFE-4BD0-8ABC-D3B5B6E1F880}" uniqueName="11" name="Asignado a" queryTableFieldId="11" dataDxfId="48"/>
+    <tableColumn id="12" xr3:uid="{A35DA601-AB84-43F1-9914-8079DAD3A955}" uniqueName="12" name="Clasificación requerimiento" queryTableFieldId="12" dataDxfId="47"/>
+    <tableColumn id="13" xr3:uid="{C9B9BAF0-055B-416F-A5B2-65E763015FD7}" uniqueName="13" name="Subdirección solicitante" queryTableFieldId="13" dataDxfId="46"/>
+    <tableColumn id="14" xr3:uid="{BC3DDA39-962F-4573-996E-77BD8BE40FB6}" uniqueName="14" name="Prioridad Origen" queryTableFieldId="14" dataDxfId="45"/>
+    <tableColumn id="15" xr3:uid="{8BE5F5D0-62C5-4ABC-BF0B-A948639C8D12}" uniqueName="15" name="F.Inicio base" queryTableFieldId="15" dataDxfId="44"/>
+    <tableColumn id="16" xr3:uid="{390C035A-E22A-4A22-8A40-84D899F95E4B}" uniqueName="16" name="F. fin base" queryTableFieldId="16" dataDxfId="43"/>
+    <tableColumn id="17" xr3:uid="{7A05EABF-0116-4EB6-8560-5EBF9F6F108B}" uniqueName="17" name="Fase" queryTableFieldId="17" dataDxfId="42"/>
+    <tableColumn id="18" xr3:uid="{7EF58F9F-F423-4B0E-AAC3-480E0531EF0C}" uniqueName="18" name="Edo. Salud" queryTableFieldId="18" dataDxfId="41"/>
+    <tableColumn id="19" xr3:uid="{A62386F7-0F54-49A2-86AC-75CB742CADA8}" uniqueName="19" name="Área Responsable Habilitación" queryTableFieldId="19" dataDxfId="40"/>
     <tableColumn id="20" xr3:uid="{A3E66536-269E-46F3-A619-26C00AA866C1}" uniqueName="20" name="Prioridad EPT" queryTableFieldId="20"/>
-    <tableColumn id="21" xr3:uid="{668E900F-B414-4186-9464-7ED7FBFACBA0}" uniqueName="21" name="Consultor de Negocio" queryTableFieldId="21" dataDxfId="41"/>
-    <tableColumn id="22" xr3:uid="{059D6A3E-BF23-4299-8B54-D5C75587AC00}" uniqueName="22" name="F Inicio Entendimiento" queryTableFieldId="22" dataDxfId="40"/>
-    <tableColumn id="23" xr3:uid="{E470E294-1EBE-49B4-9278-1132AEF3570B}" uniqueName="23" name="F Fin Entendimiento" queryTableFieldId="23" dataDxfId="39"/>
-    <tableColumn id="24" xr3:uid="{89C67E88-8FDD-49F0-8AB1-7D57BC26BEE8}" uniqueName="24" name="F Inicio Habilitación" queryTableFieldId="24" dataDxfId="38"/>
-    <tableColumn id="25" xr3:uid="{B9D22A6B-1E66-40DE-BD66-170A63B6E97E}" uniqueName="25" name="F Fin Habilitación" queryTableFieldId="25" dataDxfId="37"/>
+    <tableColumn id="21" xr3:uid="{668E900F-B414-4186-9464-7ED7FBFACBA0}" uniqueName="21" name="Consultor de Negocio" queryTableFieldId="21" dataDxfId="39"/>
+    <tableColumn id="22" xr3:uid="{059D6A3E-BF23-4299-8B54-D5C75587AC00}" uniqueName="22" name="F Inicio Entendimiento" queryTableFieldId="22" dataDxfId="38"/>
+    <tableColumn id="23" xr3:uid="{E470E294-1EBE-49B4-9278-1132AEF3570B}" uniqueName="23" name="F Fin Entendimiento" queryTableFieldId="23" dataDxfId="37"/>
+    <tableColumn id="24" xr3:uid="{89C67E88-8FDD-49F0-8AB1-7D57BC26BEE8}" uniqueName="24" name="F Inicio Habilitación" queryTableFieldId="24" dataDxfId="36"/>
+    <tableColumn id="25" xr3:uid="{B9D22A6B-1E66-40DE-BD66-170A63B6E97E}" uniqueName="25" name="F Fin Habilitación" queryTableFieldId="25" dataDxfId="35"/>
     <tableColumn id="26" xr3:uid="{83E5DB82-638A-43D5-96F4-A7AED7DF956A}" uniqueName="26" name="Tiempo dedicado" queryTableFieldId="26"/>
     <tableColumn id="27" xr3:uid="{15314FD9-16B1-4D52-9A30-456B38C78EE1}" uniqueName="27" name="Tiempo total dedicado" queryTableFieldId="27"/>
   </tableColumns>
@@ -2978,31 +2988,31 @@
   <autoFilter ref="A1:R63" xr:uid="{D875CE02-F7C9-4E02-A37D-8343287566A8}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{943C3F01-5D10-4FC6-9B11-6E753363D39C}" uniqueName="1" name="#" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{F00A8135-3890-4DC8-B8E1-7160A561B4F7}" uniqueName="2" name="Grupo de tarea" queryTableFieldId="2" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{C69CF7E3-D0AE-4ED2-BFBD-FC2F4F1532AF}" uniqueName="3" name="Asignado a" queryTableFieldId="3" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{B53BF107-D92B-4CBA-B810-160097A7A588}" uniqueName="4" name="Asunto" queryTableFieldId="4" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{DA650B1D-1F40-49DF-BB18-B735BDBFDC7F}" uniqueName="5" name="Estado" queryTableFieldId="5" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{F00A8135-3890-4DC8-B8E1-7160A561B4F7}" uniqueName="2" name="Grupo de tarea" queryTableFieldId="2" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{C69CF7E3-D0AE-4ED2-BFBD-FC2F4F1532AF}" uniqueName="3" name="Asignado a" queryTableFieldId="3" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{B53BF107-D92B-4CBA-B810-160097A7A588}" uniqueName="4" name="Asunto" queryTableFieldId="4" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{DA650B1D-1F40-49DF-BB18-B735BDBFDC7F}" uniqueName="5" name="Estado" queryTableFieldId="5" dataDxfId="31"/>
     <tableColumn id="6" xr3:uid="{56B26D9E-76A9-418C-A957-C9A83F2A3B9D}" uniqueName="6" name="Prioridad EPT" queryTableFieldId="6"/>
-    <tableColumn id="7" xr3:uid="{76F217D5-4C6D-42AE-8669-C80750F2F73B}" uniqueName="7" name="Fase" queryTableFieldId="7" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{6EFB5032-28F9-4E10-BE0A-203AA84FD3AF}" uniqueName="8" name="Impacto de Otros Proyectos" queryTableFieldId="8" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{76654024-67C4-4DAD-B036-95E06B9FEE5A}" uniqueName="9" name="Capacidades" queryTableFieldId="9" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{05F5B258-1AA7-466C-9D71-13E6BF6881D7}" uniqueName="10" name="Acciones Coordinadas STI" queryTableFieldId="10" dataDxfId="29"/>
-    <tableColumn id="11" xr3:uid="{B9E89F0D-496C-4B6D-90B9-1A739109378D}" uniqueName="11" name="F.Inicio base" queryTableFieldId="11" dataDxfId="28"/>
-    <tableColumn id="12" xr3:uid="{ECA9EB3E-8499-4FF9-A4ED-23599C189D81}" uniqueName="12" name="F. fin base" queryTableFieldId="12" dataDxfId="27"/>
-    <tableColumn id="13" xr3:uid="{570B8D0D-55D1-4470-A316-1E5C514374D0}" uniqueName="13" name="Área Responsable Habilitación" queryTableFieldId="13" dataDxfId="26"/>
-    <tableColumn id="14" xr3:uid="{8C5A459F-4123-483B-BD34-742A4E00EE1D}" uniqueName="14" name="Area Apoyo Habilitación" queryTableFieldId="14" dataDxfId="25"/>
-    <tableColumn id="15" xr3:uid="{2309E18A-EBA4-473A-8898-26BCEDE037C3}" uniqueName="15" name="Tipo de Proyecto" queryTableFieldId="15" dataDxfId="24"/>
-    <tableColumn id="16" xr3:uid="{12D3379E-DF9D-47A8-93A7-BBDF0834DE21}" uniqueName="16" name="Categoría del Proyecto" queryTableFieldId="16" dataDxfId="23"/>
-    <tableColumn id="17" xr3:uid="{3627F888-9FD1-47AA-AD7F-6C7E3F30CD4E}" uniqueName="17" name="Fuente Negocio" queryTableFieldId="17" dataDxfId="22"/>
-    <tableColumn id="18" xr3:uid="{6E0C5BCC-59F6-46FF-9BA6-FD3B7150A288}" uniqueName="18" name="Fábrica Software" queryTableFieldId="18" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{76F217D5-4C6D-42AE-8669-C80750F2F73B}" uniqueName="7" name="Fase" queryTableFieldId="7" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{6EFB5032-28F9-4E10-BE0A-203AA84FD3AF}" uniqueName="8" name="Impacto de Otros Proyectos" queryTableFieldId="8" dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{76654024-67C4-4DAD-B036-95E06B9FEE5A}" uniqueName="9" name="Capacidades" queryTableFieldId="9" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{05F5B258-1AA7-466C-9D71-13E6BF6881D7}" uniqueName="10" name="Acciones Coordinadas STI" queryTableFieldId="10" dataDxfId="27"/>
+    <tableColumn id="11" xr3:uid="{B9E89F0D-496C-4B6D-90B9-1A739109378D}" uniqueName="11" name="F.Inicio base" queryTableFieldId="11" dataDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{ECA9EB3E-8499-4FF9-A4ED-23599C189D81}" uniqueName="12" name="F. fin base" queryTableFieldId="12" dataDxfId="25"/>
+    <tableColumn id="13" xr3:uid="{570B8D0D-55D1-4470-A316-1E5C514374D0}" uniqueName="13" name="Área Responsable Habilitación" queryTableFieldId="13" dataDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{8C5A459F-4123-483B-BD34-742A4E00EE1D}" uniqueName="14" name="Area Apoyo Habilitación" queryTableFieldId="14" dataDxfId="23"/>
+    <tableColumn id="15" xr3:uid="{2309E18A-EBA4-473A-8898-26BCEDE037C3}" uniqueName="15" name="Tipo de Proyecto" queryTableFieldId="15" dataDxfId="22"/>
+    <tableColumn id="16" xr3:uid="{12D3379E-DF9D-47A8-93A7-BBDF0834DE21}" uniqueName="16" name="Categoría del Proyecto" queryTableFieldId="16" dataDxfId="21"/>
+    <tableColumn id="17" xr3:uid="{3627F888-9FD1-47AA-AD7F-6C7E3F30CD4E}" uniqueName="17" name="Fuente Negocio" queryTableFieldId="17" dataDxfId="20"/>
+    <tableColumn id="18" xr3:uid="{6E0C5BCC-59F6-46FF-9BA6-FD3B7150A288}" uniqueName="18" name="Fábrica Software" queryTableFieldId="18" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1356BC0B-6CFE-43EF-A014-6B5BFB770976}" name="Tabla5" displayName="Tabla5" ref="A1:M50" totalsRowShown="0">
-  <autoFilter ref="A1:M50" xr:uid="{1356BC0B-6CFE-43EF-A014-6B5BFB770976}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{1356BC0B-6CFE-43EF-A014-6B5BFB770976}" name="Tabla5" displayName="Tabla5" ref="A1:M52" totalsRowShown="0">
+  <autoFilter ref="A1:M52" xr:uid="{1356BC0B-6CFE-43EF-A014-6B5BFB770976}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{F090BF8D-B2F7-4580-A229-645DDC1BF7E7}" name="#"/>
     <tableColumn id="2" xr3:uid="{19A6B4EC-A68B-4D61-ADC4-7FA329BF3F2D}" name="Grupo de tarea"/>
@@ -3010,8 +3020,8 @@
     <tableColumn id="4" xr3:uid="{04384FA7-53FA-4216-9E4E-7DAD8FE57F3D}" name="DO"/>
     <tableColumn id="5" xr3:uid="{1380DC78-BE61-4674-BD0B-B2347BD7AF71}" name="Fase"/>
     <tableColumn id="6" xr3:uid="{F46844C4-7998-4EFC-8EC6-3AD18A7B0C99}" name="Estado"/>
-    <tableColumn id="7" xr3:uid="{CB06D83C-0068-469B-A794-CB5995863AF3}" name="F.Inicio base" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{91304FB9-6CD1-443B-83A2-038CAC44A38F}" name="F. fin base" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{CB06D83C-0068-469B-A794-CB5995863AF3}" name="F.Inicio base" dataDxfId="57"/>
+    <tableColumn id="8" xr3:uid="{91304FB9-6CD1-443B-83A2-038CAC44A38F}" name="F. fin base" dataDxfId="56"/>
     <tableColumn id="9" xr3:uid="{F52F529B-90C9-41AE-A1EA-349DA8441A4F}" name="Situación actual"/>
     <tableColumn id="10" xr3:uid="{A1BA5E88-4A99-4870-A1AB-82B7B1D1BBF8}" name="Área Responsable Habilitación"/>
     <tableColumn id="11" xr3:uid="{4DFB4F04-67EF-43ED-AD9D-2402E2583582}" name="Resumen Acciones "/>
@@ -3027,25 +3037,25 @@
   <autoFilter ref="A1:T149" xr:uid="{9453EF90-F91B-4433-940A-9F91B8434FC4}"/>
   <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{14CEF807-9B34-4C3E-B5C6-82257C887758}" uniqueName="1" name="#" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{E0F2F729-9E65-45E6-BA2D-8F362E5ADFE1}" uniqueName="2" name="Estado" queryTableFieldId="2" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{D02EBEAA-8EB3-4C69-8A65-826D3DF33D45}" uniqueName="3" name="Asunto" queryTableFieldId="3" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{170DE0A7-E030-43CF-8D5F-ECE7AD0B503F}" uniqueName="4" name="Asignado a" queryTableFieldId="4" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{8C17A05F-3747-46CD-AF20-FDD63175735B}" uniqueName="5" name="Clasificación requerimiento" queryTableFieldId="5" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{9FDEEF2F-2683-45BA-B72A-3F72C4DF8414}" uniqueName="6" name="Grupo de tarea" queryTableFieldId="6" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{D9ED4921-DC5F-4525-95BD-01FF11E34B8D}" uniqueName="7" name="Prioridad Negocio" queryTableFieldId="7" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{B957CD1B-CB24-4E0A-A6D8-D689187C1F28}" uniqueName="8" name="Fecha de inicio" queryTableFieldId="8" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{AA7248E1-A86D-4A90-BA23-53F778872367}" uniqueName="9" name="Impacto de Otros Proyectos" queryTableFieldId="9" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{3B9B35BC-23F0-42D2-BEE2-AD63C98BFF67}" uniqueName="10" name="Capacidades" queryTableFieldId="10" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{B58D7C68-57C3-4E6B-ACBD-3C7F612737C7}" uniqueName="11" name="Acciones Coordinadas STI" queryTableFieldId="11" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{3991FC41-33BD-47AC-AD3C-18EF07F8BF76}" uniqueName="12" name="F.Inicio base" queryTableFieldId="12" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{5B8B4B94-CE37-4952-8AD4-35129F6E6CB1}" uniqueName="13" name="Fase" queryTableFieldId="13" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{07995378-FD23-4466-A1D1-DA998D1C4703}" uniqueName="14" name="Edo. Salud" queryTableFieldId="14" dataDxfId="8"/>
-    <tableColumn id="15" xr3:uid="{9D6D87E6-45BA-4937-B8A6-D740BE4D66BB}" uniqueName="15" name="Área Responsable Habilitación" queryTableFieldId="15" dataDxfId="7"/>
-    <tableColumn id="16" xr3:uid="{E65DDAEC-EFA9-4CAC-93CF-B578CF73C3AA}" uniqueName="16" name="Fuente Negocio" queryTableFieldId="16" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{65BA016F-97E7-449F-82DF-02A542B13C1D}" uniqueName="17" name="Prioridad EPT" queryTableFieldId="17" dataDxfId="5"/>
-    <tableColumn id="18" xr3:uid="{EC5EA07C-6DA8-4187-94F8-0C9257AB86CE}" uniqueName="18" name="Consultor de Negocio" queryTableFieldId="18" dataDxfId="4"/>
-    <tableColumn id="19" xr3:uid="{51357594-1D35-4BED-97A1-793ABA0EAA2B}" uniqueName="19" name="F Inicio Entendimiento" queryTableFieldId="19" dataDxfId="3"/>
-    <tableColumn id="20" xr3:uid="{DCCCE3AF-8188-492B-AE44-753E558A2552}" uniqueName="20" name="F Fin Entendimiento" queryTableFieldId="20" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{E0F2F729-9E65-45E6-BA2D-8F362E5ADFE1}" uniqueName="2" name="Estado" queryTableFieldId="2" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{D02EBEAA-8EB3-4C69-8A65-826D3DF33D45}" uniqueName="3" name="Asunto" queryTableFieldId="3" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{170DE0A7-E030-43CF-8D5F-ECE7AD0B503F}" uniqueName="4" name="Asignado a" queryTableFieldId="4" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{8C17A05F-3747-46CD-AF20-FDD63175735B}" uniqueName="5" name="Clasificación requerimiento" queryTableFieldId="5" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{9FDEEF2F-2683-45BA-B72A-3F72C4DF8414}" uniqueName="6" name="Grupo de tarea" queryTableFieldId="6" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{D9ED4921-DC5F-4525-95BD-01FF11E34B8D}" uniqueName="7" name="Prioridad Negocio" queryTableFieldId="7" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{B957CD1B-CB24-4E0A-A6D8-D689187C1F28}" uniqueName="8" name="Fecha de inicio" queryTableFieldId="8" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{AA7248E1-A86D-4A90-BA23-53F778872367}" uniqueName="9" name="Impacto de Otros Proyectos" queryTableFieldId="9" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{3B9B35BC-23F0-42D2-BEE2-AD63C98BFF67}" uniqueName="10" name="Capacidades" queryTableFieldId="10" dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{B58D7C68-57C3-4E6B-ACBD-3C7F612737C7}" uniqueName="11" name="Acciones Coordinadas STI" queryTableFieldId="11" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{3991FC41-33BD-47AC-AD3C-18EF07F8BF76}" uniqueName="12" name="F.Inicio base" queryTableFieldId="12" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{5B8B4B94-CE37-4952-8AD4-35129F6E6CB1}" uniqueName="13" name="Fase" queryTableFieldId="13" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{07995378-FD23-4466-A1D1-DA998D1C4703}" uniqueName="14" name="Edo. Salud" queryTableFieldId="14" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{9D6D87E6-45BA-4937-B8A6-D740BE4D66BB}" uniqueName="15" name="Área Responsable Habilitación" queryTableFieldId="15" dataDxfId="5"/>
+    <tableColumn id="16" xr3:uid="{E65DDAEC-EFA9-4CAC-93CF-B578CF73C3AA}" uniqueName="16" name="Fuente Negocio" queryTableFieldId="16" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{65BA016F-97E7-449F-82DF-02A542B13C1D}" uniqueName="17" name="Prioridad EPT" queryTableFieldId="17" dataDxfId="3"/>
+    <tableColumn id="18" xr3:uid="{EC5EA07C-6DA8-4187-94F8-0C9257AB86CE}" uniqueName="18" name="Consultor de Negocio" queryTableFieldId="18" dataDxfId="2"/>
+    <tableColumn id="19" xr3:uid="{51357594-1D35-4BED-97A1-793ABA0EAA2B}" uniqueName="19" name="F Inicio Entendimiento" queryTableFieldId="19" dataDxfId="1"/>
+    <tableColumn id="20" xr3:uid="{DCCCE3AF-8188-492B-AE44-753E558A2552}" uniqueName="20" name="F Fin Entendimiento" queryTableFieldId="20" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3369,36 +3379,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F4782CA-7A9A-4EAF-A3C3-A0ABE6859531}">
   <dimension ref="A1:AA100"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="81.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="81.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="81.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="81.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="33.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.90625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="78" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="32.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="31.109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="26" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="32.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="31.08984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="29.6328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="23.90625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="25" max="26" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="23.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3481,7 +3491,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>120063</v>
       </c>
@@ -3553,7 +3563,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>120039</v>
       </c>
@@ -3625,7 +3635,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>119355</v>
       </c>
@@ -3700,7 +3710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>119234</v>
       </c>
@@ -3775,7 +3785,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>118980</v>
       </c>
@@ -3850,7 +3860,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>118945</v>
       </c>
@@ -3925,7 +3935,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>118801</v>
       </c>
@@ -3994,7 +4004,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>118771</v>
       </c>
@@ -4063,7 +4073,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>118752</v>
       </c>
@@ -4138,7 +4148,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>118736</v>
       </c>
@@ -4217,7 +4227,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>118715</v>
       </c>
@@ -4298,7 +4308,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>118679</v>
       </c>
@@ -4377,7 +4387,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>118656</v>
       </c>
@@ -4455,7 +4465,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>118621</v>
       </c>
@@ -4533,7 +4543,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>118558</v>
       </c>
@@ -4603,7 +4613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>118506</v>
       </c>
@@ -4678,7 +4688,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>118487</v>
       </c>
@@ -4753,7 +4763,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>118463</v>
       </c>
@@ -4834,7 +4844,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>118402</v>
       </c>
@@ -4917,7 +4927,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>118383</v>
       </c>
@@ -4990,7 +5000,7 @@
         <v>6600</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>118334</v>
       </c>
@@ -5073,7 +5083,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>118265</v>
       </c>
@@ -5149,7 +5159,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>117731</v>
       </c>
@@ -5230,7 +5240,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>117647</v>
       </c>
@@ -5306,7 +5316,7 @@
         <v>4820</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>117591</v>
       </c>
@@ -5378,7 +5388,7 @@
         <v>2900</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>117534</v>
       </c>
@@ -5457,7 +5467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>117508</v>
       </c>
@@ -5536,7 +5546,7 @@
         <v>19600</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>117480</v>
       </c>
@@ -5614,7 +5624,7 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>117422</v>
       </c>
@@ -5693,7 +5703,7 @@
         <v>20300</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>117235</v>
       </c>
@@ -5776,7 +5786,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>117234</v>
       </c>
@@ -5859,7 +5869,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>117132</v>
       </c>
@@ -5938,7 +5948,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>116948</v>
       </c>
@@ -6014,7 +6024,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>116844</v>
       </c>
@@ -6093,7 +6103,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>116827</v>
       </c>
@@ -6168,7 +6178,7 @@
         <v>40000</v>
       </c>
     </row>
-    <row r="37" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>115921</v>
       </c>
@@ -6251,7 +6261,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="38" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>115850</v>
       </c>
@@ -6332,7 +6342,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="39" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>115794</v>
       </c>
@@ -6415,7 +6425,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="40" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>115772</v>
       </c>
@@ -6498,7 +6508,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="41" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>115745</v>
       </c>
@@ -6579,7 +6589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>115684</v>
       </c>
@@ -6660,7 +6670,7 @@
         <v>7800</v>
       </c>
     </row>
-    <row r="43" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>115661</v>
       </c>
@@ -6735,7 +6745,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="44" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>115393</v>
       </c>
@@ -6810,7 +6820,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="45" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>115350</v>
       </c>
@@ -6893,7 +6903,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="46" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>115296</v>
       </c>
@@ -6976,7 +6986,7 @@
         <v>11100</v>
       </c>
     </row>
-    <row r="47" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>115066</v>
       </c>
@@ -7059,7 +7069,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="48" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>115050</v>
       </c>
@@ -7142,7 +7152,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="49" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>114802</v>
       </c>
@@ -7225,7 +7235,7 @@
         <v>11800</v>
       </c>
     </row>
-    <row r="50" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>114703</v>
       </c>
@@ -7300,7 +7310,7 @@
         <v>35430</v>
       </c>
     </row>
-    <row r="51" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>114317</v>
       </c>
@@ -7379,7 +7389,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>114283</v>
       </c>
@@ -7458,7 +7468,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>113973</v>
       </c>
@@ -7536,7 +7546,7 @@
         <v>9300</v>
       </c>
     </row>
-    <row r="54" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>113886</v>
       </c>
@@ -7615,7 +7625,7 @@
         <v>51500</v>
       </c>
     </row>
-    <row r="55" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>113629</v>
       </c>
@@ -7687,7 +7697,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="56" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>112732</v>
       </c>
@@ -7770,7 +7780,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="57" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>112410</v>
       </c>
@@ -7849,7 +7859,7 @@
         <v>21000</v>
       </c>
     </row>
-    <row r="58" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>112320</v>
       </c>
@@ -7928,7 +7938,7 @@
         <v>14125</v>
       </c>
     </row>
-    <row r="59" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>110891</v>
       </c>
@@ -8007,7 +8017,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="60" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>110615</v>
       </c>
@@ -8082,7 +8092,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="61" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>110247</v>
       </c>
@@ -8163,7 +8173,7 @@
         <v>10780</v>
       </c>
     </row>
-    <row r="62" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>109795</v>
       </c>
@@ -8242,7 +8252,7 @@
         <v>14200</v>
       </c>
     </row>
-    <row r="63" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>109515</v>
       </c>
@@ -8321,7 +8331,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="64" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>109472</v>
       </c>
@@ -8402,7 +8412,7 @@
         <v>8700</v>
       </c>
     </row>
-    <row r="65" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>109358</v>
       </c>
@@ -8483,7 +8493,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="66" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>109277</v>
       </c>
@@ -8562,7 +8572,7 @@
         <v>1450</v>
       </c>
     </row>
-    <row r="67" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>109260</v>
       </c>
@@ -8643,7 +8653,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="68" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>107446</v>
       </c>
@@ -8726,7 +8736,7 @@
         <v>1830</v>
       </c>
     </row>
-    <row r="69" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>107352</v>
       </c>
@@ -8805,7 +8815,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="70" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>106611</v>
       </c>
@@ -8880,7 +8890,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="71" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>106316</v>
       </c>
@@ -8955,7 +8965,7 @@
         <v>1310</v>
       </c>
     </row>
-    <row r="72" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>106154</v>
       </c>
@@ -9034,7 +9044,7 @@
         <v>12015</v>
       </c>
     </row>
-    <row r="73" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>105760</v>
       </c>
@@ -9115,7 +9125,7 @@
         <v>7500</v>
       </c>
     </row>
-    <row r="74" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>105704</v>
       </c>
@@ -9194,7 +9204,7 @@
         <v>12400</v>
       </c>
     </row>
-    <row r="75" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>105614</v>
       </c>
@@ -9273,7 +9283,7 @@
         <v>2125</v>
       </c>
     </row>
-    <row r="76" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>105530</v>
       </c>
@@ -9349,7 +9359,7 @@
         <v>1345</v>
       </c>
     </row>
-    <row r="77" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>105432</v>
       </c>
@@ -9425,7 +9435,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="78" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>105030</v>
       </c>
@@ -9508,7 +9518,7 @@
         <v>3900</v>
       </c>
     </row>
-    <row r="79" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>103458</v>
       </c>
@@ -9588,7 +9598,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="80" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>102966</v>
       </c>
@@ -9669,7 +9679,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="81" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>102945</v>
       </c>
@@ -9752,7 +9762,7 @@
         <v>18600</v>
       </c>
     </row>
-    <row r="82" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>102600</v>
       </c>
@@ -9829,7 +9839,7 @@
         <v>21190</v>
       </c>
     </row>
-    <row r="83" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>102323</v>
       </c>
@@ -9908,7 +9918,7 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="84" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>102164</v>
       </c>
@@ -9987,7 +9997,7 @@
         <v>5480</v>
       </c>
     </row>
-    <row r="85" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>101074</v>
       </c>
@@ -10062,7 +10072,7 @@
         <v>4340</v>
       </c>
     </row>
-    <row r="86" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>100384</v>
       </c>
@@ -10141,7 +10151,7 @@
         <v>1930</v>
       </c>
     </row>
-    <row r="87" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>100189</v>
       </c>
@@ -10224,7 +10234,7 @@
         <v>61950</v>
       </c>
     </row>
-    <row r="88" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>93698</v>
       </c>
@@ -10304,7 +10314,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="89" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>93318</v>
       </c>
@@ -10383,7 +10393,7 @@
         <v>4610</v>
       </c>
     </row>
-    <row r="90" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>93189</v>
       </c>
@@ -10463,7 +10473,7 @@
         <v>2810</v>
       </c>
     </row>
-    <row r="91" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>90975</v>
       </c>
@@ -10542,7 +10552,7 @@
         <v>17540</v>
       </c>
     </row>
-    <row r="92" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>89593</v>
       </c>
@@ -10617,7 +10627,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="93" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>88736</v>
       </c>
@@ -10696,7 +10706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>77906</v>
       </c>
@@ -10777,7 +10787,7 @@
         <v>8705</v>
       </c>
     </row>
-    <row r="95" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>72138</v>
       </c>
@@ -10858,7 +10868,7 @@
         <v>61750</v>
       </c>
     </row>
-    <row r="96" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>69537</v>
       </c>
@@ -10941,7 +10951,7 @@
         <v>55550</v>
       </c>
     </row>
-    <row r="97" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>52391</v>
       </c>
@@ -11024,7 +11034,7 @@
         <v>6545</v>
       </c>
     </row>
-    <row r="98" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>50889</v>
       </c>
@@ -11101,7 +11111,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="99" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>47608</v>
       </c>
@@ -11180,7 +11190,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="100" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>46211</v>
       </c>
@@ -11274,29 +11284,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7962065-83B7-4F84-AE15-90C9DE0413AD}">
   <dimension ref="A1:R63"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="81.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="81.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="31.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="81.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="81.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31.08984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.453125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="49" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="31" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -11352,7 +11362,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>115154</v>
       </c>
@@ -11406,7 +11416,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>112090</v>
       </c>
@@ -11460,7 +11470,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>111287</v>
       </c>
@@ -11514,7 +11524,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>110745</v>
       </c>
@@ -11568,7 +11578,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>110439</v>
       </c>
@@ -11622,7 +11632,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>108568</v>
       </c>
@@ -11676,7 +11686,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>107319</v>
       </c>
@@ -11730,7 +11740,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>107285</v>
       </c>
@@ -11784,7 +11794,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>107269</v>
       </c>
@@ -11838,7 +11848,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>107096</v>
       </c>
@@ -11892,7 +11902,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>106902</v>
       </c>
@@ -11946,7 +11956,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>105361</v>
       </c>
@@ -12000,7 +12010,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>104964</v>
       </c>
@@ -12054,7 +12064,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>103395</v>
       </c>
@@ -12105,7 +12115,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>103206</v>
       </c>
@@ -12159,7 +12169,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>102564</v>
       </c>
@@ -12210,7 +12220,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>100015</v>
       </c>
@@ -12264,7 +12274,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>97394</v>
       </c>
@@ -12318,7 +12328,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>97136</v>
       </c>
@@ -12369,7 +12379,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>92135</v>
       </c>
@@ -12420,7 +12430,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>90064</v>
       </c>
@@ -12474,7 +12484,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>90004</v>
       </c>
@@ -12528,7 +12538,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>88939</v>
       </c>
@@ -12582,7 +12592,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>88806</v>
       </c>
@@ -12636,7 +12646,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>86728</v>
       </c>
@@ -12690,7 +12700,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>84529</v>
       </c>
@@ -12744,7 +12754,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>83846</v>
       </c>
@@ -12798,7 +12808,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>83175</v>
       </c>
@@ -12852,7 +12862,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>81795</v>
       </c>
@@ -12906,7 +12916,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>80951</v>
       </c>
@@ -12957,7 +12967,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>80842</v>
       </c>
@@ -13011,7 +13021,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>79160</v>
       </c>
@@ -13065,7 +13075,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>78607</v>
       </c>
@@ -13119,7 +13129,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>77244</v>
       </c>
@@ -13173,7 +13183,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>77069</v>
       </c>
@@ -13227,7 +13237,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>76848</v>
       </c>
@@ -13281,7 +13291,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>76830</v>
       </c>
@@ -13335,7 +13345,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>76486</v>
       </c>
@@ -13389,7 +13399,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>70262</v>
       </c>
@@ -13445,7 +13455,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>65489</v>
       </c>
@@ -13499,7 +13509,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>62403</v>
       </c>
@@ -13550,7 +13560,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>62048</v>
       </c>
@@ -13604,7 +13614,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>61095</v>
       </c>
@@ -13658,7 +13668,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>60657</v>
       </c>
@@ -13712,7 +13722,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>60149</v>
       </c>
@@ -13763,7 +13773,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>59834</v>
       </c>
@@ -13817,7 +13827,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>58368</v>
       </c>
@@ -13871,7 +13881,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>58145</v>
       </c>
@@ -13922,7 +13932,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>57980</v>
       </c>
@@ -13976,7 +13986,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>53406</v>
       </c>
@@ -14030,7 +14040,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51988</v>
       </c>
@@ -14081,7 +14091,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>51819</v>
       </c>
@@ -14135,7 +14145,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>50733</v>
       </c>
@@ -14189,7 +14199,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>49240</v>
       </c>
@@ -14243,7 +14253,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>49220</v>
       </c>
@@ -14294,7 +14304,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>48275</v>
       </c>
@@ -14348,7 +14358,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>45907</v>
       </c>
@@ -14402,7 +14412,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>45722</v>
       </c>
@@ -14453,7 +14463,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>43235</v>
       </c>
@@ -14507,7 +14517,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>32461</v>
       </c>
@@ -14558,7 +14568,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>16843</v>
       </c>
@@ -14609,7 +14619,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>15369</v>
       </c>
@@ -14673,19 +14683,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA197159-6353-47D4-9EAA-1795E713D028}">
-  <dimension ref="A1:M50"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M52"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="15.109375" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" customWidth="1"/>
-    <col min="10" max="10" width="28.33203125" customWidth="1"/>
-    <col min="11" max="11" width="18.77734375" customWidth="1"/>
-    <col min="12" max="12" width="15.6640625" customWidth="1"/>
-    <col min="13" max="13" width="16.88671875" customWidth="1"/>
+    <col min="2" max="2" width="15.08984375" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" customWidth="1"/>
+    <col min="9" max="9" width="16.36328125" customWidth="1"/>
+    <col min="10" max="10" width="28.36328125" customWidth="1"/>
+    <col min="11" max="11" width="18.81640625" customWidth="1"/>
+    <col min="12" max="12" width="15.6328125" customWidth="1"/>
+    <col min="13" max="13" width="16.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -14726,7 +14736,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>117561</v>
       </c>
@@ -14767,7 +14777,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>117175</v>
       </c>
@@ -14808,7 +14818,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>117091</v>
       </c>
@@ -14849,7 +14859,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>116806</v>
       </c>
@@ -14887,7 +14897,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>116548</v>
       </c>
@@ -14928,7 +14938,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>116317</v>
       </c>
@@ -14969,7 +14979,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>116215</v>
       </c>
@@ -15010,7 +15020,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>115700</v>
       </c>
@@ -15051,7 +15061,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>115547</v>
       </c>
@@ -15092,7 +15102,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>115481</v>
       </c>
@@ -15133,7 +15143,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>115188</v>
       </c>
@@ -15174,7 +15184,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>115172</v>
       </c>
@@ -15215,7 +15225,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>114876</v>
       </c>
@@ -15256,7 +15266,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>114744</v>
       </c>
@@ -15297,7 +15307,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>114658</v>
       </c>
@@ -15338,7 +15348,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>114228</v>
       </c>
@@ -15379,7 +15389,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>113554</v>
       </c>
@@ -15420,7 +15430,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>113506</v>
       </c>
@@ -15461,7 +15471,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>112839</v>
       </c>
@@ -15502,7 +15512,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>112786</v>
       </c>
@@ -15543,7 +15553,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>112769</v>
       </c>
@@ -15584,7 +15594,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>112748</v>
       </c>
@@ -15625,7 +15635,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>112613</v>
       </c>
@@ -15666,7 +15676,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>112118</v>
       </c>
@@ -15707,7 +15717,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>112051</v>
       </c>
@@ -15748,7 +15758,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>111374</v>
       </c>
@@ -15786,7 +15796,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>111304</v>
       </c>
@@ -15827,7 +15837,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>111009</v>
       </c>
@@ -15868,7 +15878,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>110806</v>
       </c>
@@ -15909,7 +15919,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>110789</v>
       </c>
@@ -15950,7 +15960,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>110729</v>
       </c>
@@ -15991,7 +16001,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>110101</v>
       </c>
@@ -16032,7 +16042,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>109991</v>
       </c>
@@ -16073,7 +16083,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>108618</v>
       </c>
@@ -16114,7 +16124,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>107948</v>
       </c>
@@ -16155,7 +16165,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>107480</v>
       </c>
@@ -16196,7 +16206,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>107349</v>
       </c>
@@ -16234,7 +16244,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>107230</v>
       </c>
@@ -16275,7 +16285,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>107147</v>
       </c>
@@ -16316,7 +16326,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>106433</v>
       </c>
@@ -16357,7 +16367,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>106188</v>
       </c>
@@ -16398,7 +16408,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>102878</v>
       </c>
@@ -16439,7 +16449,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>102753</v>
       </c>
@@ -16480,7 +16490,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>94198</v>
       </c>
@@ -16521,7 +16531,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>92779</v>
       </c>
@@ -16562,7 +16572,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>91996</v>
       </c>
@@ -16603,7 +16613,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>85060</v>
       </c>
@@ -16644,7 +16654,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>58384</v>
       </c>
@@ -16682,7 +16692,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>55223</v>
       </c>
@@ -16720,6 +16730,88 @@
         <v>373</v>
       </c>
       <c r="M50" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>19999</v>
+      </c>
+      <c r="B51" t="s">
+        <v>456</v>
+      </c>
+      <c r="C51" t="s">
+        <v>760</v>
+      </c>
+      <c r="D51">
+        <v>2020</v>
+      </c>
+      <c r="E51" t="s">
+        <v>101</v>
+      </c>
+      <c r="F51" t="s">
+        <v>124</v>
+      </c>
+      <c r="G51" s="3">
+        <v>44389</v>
+      </c>
+      <c r="H51" s="3">
+        <v>46079</v>
+      </c>
+      <c r="I51" t="s">
+        <v>544</v>
+      </c>
+      <c r="J51" t="s">
+        <v>41</v>
+      </c>
+      <c r="K51" t="s">
+        <v>31</v>
+      </c>
+      <c r="L51" t="s">
+        <v>373</v>
+      </c>
+      <c r="M51" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>91199</v>
+      </c>
+      <c r="B52" t="s">
+        <v>456</v>
+      </c>
+      <c r="C52" t="s">
+        <v>761</v>
+      </c>
+      <c r="D52">
+        <v>2020</v>
+      </c>
+      <c r="E52" t="s">
+        <v>101</v>
+      </c>
+      <c r="F52" t="s">
+        <v>124</v>
+      </c>
+      <c r="G52" s="3">
+        <v>44389</v>
+      </c>
+      <c r="H52" s="3">
+        <v>46079</v>
+      </c>
+      <c r="I52" t="s">
+        <v>544</v>
+      </c>
+      <c r="J52" t="s">
+        <v>41</v>
+      </c>
+      <c r="K52" t="s">
+        <v>31</v>
+      </c>
+      <c r="L52" t="s">
+        <v>373</v>
+      </c>
+      <c r="M52" t="s">
         <v>31</v>
       </c>
     </row>
@@ -16734,31 +16826,31 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC147D97-9B2A-47D1-AA7E-F2BB0D9CB615}">
   <dimension ref="A1:T149"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="81.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="81.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="31.109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="81.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="31.08984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.08984375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="23" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.90625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="21.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -16820,7 +16912,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>118586</v>
       </c>
@@ -16882,7 +16974,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>118585</v>
       </c>
@@ -16944,7 +17036,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>119453</v>
       </c>
@@ -17006,7 +17098,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>73227</v>
       </c>
@@ -17068,7 +17160,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>114316</v>
       </c>
@@ -17130,7 +17222,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>109465</v>
       </c>
@@ -17192,7 +17284,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>54566</v>
       </c>
@@ -17254,7 +17346,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>74091</v>
       </c>
@@ -17316,7 +17408,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>91700</v>
       </c>
@@ -17378,7 +17470,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>82910</v>
       </c>
@@ -17440,7 +17532,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>110614</v>
       </c>
@@ -17502,7 +17594,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>77898</v>
       </c>
@@ -17564,7 +17656,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>113245</v>
       </c>
@@ -17626,7 +17718,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>54565</v>
       </c>
@@ -17688,7 +17780,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>49817</v>
       </c>
@@ -17750,7 +17842,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>89825</v>
       </c>
@@ -17812,7 +17904,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>87031</v>
       </c>
@@ -17874,7 +17966,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>99014</v>
       </c>
@@ -17936,7 +18028,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>50014</v>
       </c>
@@ -17998,7 +18090,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>48809</v>
       </c>
@@ -18060,7 +18152,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>115295</v>
       </c>
@@ -18122,7 +18214,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>109466</v>
       </c>
@@ -18184,7 +18276,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>76687</v>
       </c>
@@ -18246,7 +18338,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>51230</v>
       </c>
@@ -18308,7 +18400,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>98880</v>
       </c>
@@ -18370,7 +18462,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>86298</v>
       </c>
@@ -18432,7 +18524,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>100863</v>
       </c>
@@ -18494,7 +18586,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>76590</v>
       </c>
@@ -18556,7 +18648,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>104307</v>
       </c>
@@ -18618,7 +18710,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>110613</v>
       </c>
@@ -18680,7 +18772,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>41045</v>
       </c>
@@ -18742,7 +18834,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>113451</v>
       </c>
@@ -18804,7 +18896,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>93307</v>
       </c>
@@ -18866,7 +18958,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>106233</v>
       </c>
@@ -18928,7 +19020,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>57724</v>
       </c>
@@ -18990,7 +19082,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>61349</v>
       </c>
@@ -19052,7 +19144,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>77150</v>
       </c>
@@ -19114,7 +19206,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>93131</v>
       </c>
@@ -19176,7 +19268,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>93240</v>
       </c>
@@ -19238,7 +19330,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>92419</v>
       </c>
@@ -19300,7 +19392,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>107521</v>
       </c>
@@ -19362,7 +19454,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>107043</v>
       </c>
@@ -19424,7 +19516,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>94681</v>
       </c>
@@ -19486,7 +19578,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>102144</v>
       </c>
@@ -19548,7 +19640,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>93026</v>
       </c>
@@ -19610,7 +19702,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>115291</v>
       </c>
@@ -19672,7 +19764,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>118735</v>
       </c>
@@ -19734,7 +19826,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>118599</v>
       </c>
@@ -19796,7 +19888,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>93029</v>
       </c>
@@ -19858,7 +19950,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>108348</v>
       </c>
@@ -19920,7 +20012,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>119371</v>
       </c>
@@ -19982,7 +20074,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>106663</v>
       </c>
@@ -20044,7 +20136,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>118770</v>
       </c>
@@ -20106,7 +20198,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>118769</v>
       </c>
@@ -20168,7 +20260,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>118598</v>
       </c>
@@ -20230,7 +20322,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>107042</v>
       </c>
@@ -20292,7 +20384,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>106666</v>
       </c>
@@ -20354,7 +20446,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>112177</v>
       </c>
@@ -20416,7 +20508,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>93025</v>
       </c>
@@ -20478,7 +20570,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>109563</v>
       </c>
@@ -20540,7 +20632,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>92694</v>
       </c>
@@ -20602,7 +20694,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>120030</v>
       </c>
@@ -20664,7 +20756,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>43313</v>
       </c>
@@ -20726,7 +20818,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>114058</v>
       </c>
@@ -20788,7 +20880,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>43340</v>
       </c>
@@ -20850,7 +20942,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>103439</v>
       </c>
@@ -20912,7 +21004,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>86377</v>
       </c>
@@ -20974,7 +21066,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>99963</v>
       </c>
@@ -21036,7 +21128,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>117085</v>
       </c>
@@ -21098,7 +21190,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>63866</v>
       </c>
@@ -21160,7 +21252,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>118674</v>
       </c>
@@ -21222,7 +21314,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>110461</v>
       </c>
@@ -21284,7 +21376,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>69536</v>
       </c>
@@ -21346,7 +21438,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>76448</v>
       </c>
@@ -21408,7 +21500,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>112458</v>
       </c>
@@ -21470,7 +21562,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>92977</v>
       </c>
@@ -21532,7 +21624,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>69727</v>
       </c>
@@ -21594,7 +21686,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>46033</v>
       </c>
@@ -21656,7 +21748,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>65515</v>
       </c>
@@ -21718,7 +21810,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>116057</v>
       </c>
@@ -21780,7 +21872,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>117086</v>
       </c>
@@ -21842,7 +21934,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>117578</v>
       </c>
@@ -21904,7 +21996,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>111874</v>
       </c>
@@ -21966,7 +22058,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>111286</v>
       </c>
@@ -22028,7 +22120,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>116965</v>
       </c>
@@ -22090,7 +22182,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>119383</v>
       </c>
@@ -22152,7 +22244,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>114165</v>
       </c>
@@ -22214,7 +22306,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>112438</v>
       </c>
@@ -22276,7 +22368,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>111876</v>
       </c>
@@ -22338,7 +22430,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>114597</v>
       </c>
@@ -22400,7 +22492,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>119250</v>
       </c>
@@ -22462,7 +22554,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>118731</v>
       </c>
@@ -22524,7 +22616,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>115205</v>
       </c>
@@ -22586,7 +22678,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>118481</v>
       </c>
@@ -22648,7 +22740,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>118850</v>
       </c>
@@ -22710,7 +22802,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>118734</v>
       </c>
@@ -22772,7 +22864,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>116684</v>
       </c>
@@ -22834,7 +22926,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>114927</v>
       </c>
@@ -22896,7 +22988,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>115479</v>
       </c>
@@ -22958,7 +23050,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>112804</v>
       </c>
@@ -23020,7 +23112,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>120033</v>
       </c>
@@ -23082,7 +23174,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>111815</v>
       </c>
@@ -23144,7 +23236,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>117556</v>
       </c>
@@ -23206,7 +23298,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>118421</v>
       </c>
@@ -23268,7 +23360,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>113665</v>
       </c>
@@ -23330,7 +23422,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>113669</v>
       </c>
@@ -23392,7 +23484,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>118732</v>
       </c>
@@ -23454,7 +23546,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>90614</v>
       </c>
@@ -23516,7 +23608,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>111567</v>
       </c>
@@ -23578,7 +23670,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>114249</v>
       </c>
@@ -23640,7 +23732,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>116973</v>
       </c>
@@ -23702,7 +23794,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>113038</v>
       </c>
@@ -23764,7 +23856,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>118311</v>
       </c>
@@ -23826,7 +23918,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>112492</v>
       </c>
@@ -23888,7 +23980,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>112159</v>
       </c>
@@ -23950,7 +24042,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>118675</v>
       </c>
@@ -24012,7 +24104,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="118" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>116739</v>
       </c>
@@ -24074,7 +24166,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>94175</v>
       </c>
@@ -24136,7 +24228,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="120" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>101394</v>
       </c>
@@ -24198,7 +24290,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="121" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>114741</v>
       </c>
@@ -24260,7 +24352,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="122" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>79535</v>
       </c>
@@ -24322,7 +24414,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>109603</v>
       </c>
@@ -24384,7 +24476,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>113768</v>
       </c>
@@ -24446,7 +24538,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>114637</v>
       </c>
@@ -24508,7 +24600,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="126" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>106629</v>
       </c>
@@ -24570,7 +24662,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="127" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>94174</v>
       </c>
@@ -24632,7 +24724,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="128" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>97440</v>
       </c>
@@ -24694,7 +24786,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="129" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>101313</v>
       </c>
@@ -24756,7 +24848,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="130" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>97728</v>
       </c>
@@ -24818,7 +24910,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="131" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>101378</v>
       </c>
@@ -24880,7 +24972,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="132" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>117355</v>
       </c>
@@ -24942,7 +25034,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="133" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>74135</v>
       </c>
@@ -25004,7 +25096,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="134" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>110702</v>
       </c>
@@ -25066,7 +25158,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="135" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>110703</v>
       </c>
@@ -25128,7 +25220,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="136" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>117531</v>
       </c>
@@ -25190,7 +25282,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>99250</v>
       </c>
@@ -25252,7 +25344,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>105839</v>
       </c>
@@ -25314,7 +25406,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>81849</v>
       </c>
@@ -25376,7 +25468,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>95292</v>
       </c>
@@ -25438,7 +25530,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>85296</v>
       </c>
@@ -25500,7 +25592,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>94431</v>
       </c>
@@ -25562,7 +25654,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="143" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>100115</v>
       </c>
@@ -25624,7 +25716,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>102359</v>
       </c>
@@ -25686,7 +25778,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="145" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>85298</v>
       </c>
@@ -25748,7 +25840,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="146" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>86226</v>
       </c>
@@ -25810,7 +25902,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="147" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>66503</v>
       </c>
@@ -25872,7 +25964,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="148" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>85300</v>
       </c>
@@ -25934,7 +26026,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="149" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>109885</v>
       </c>

</xml_diff>